<commit_message>
#5 Add Risk Register/correction
</commit_message>
<xml_diff>
--- a/project-management/risks/Risk_Register_SmartParking.xlsx
+++ b/project-management/risks/Risk_Register_SmartParking.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="135">
   <si>
     <t>RISK REGISTER</t>
   </si>
@@ -253,13 +253,13 @@
     <t>Falta de disponibilidad de componentes durante la construcción</t>
   </si>
   <si>
-    <t>Retrasos o dificultades para adquirir sensores, cables u otros componentes</t>
+    <t>Retrasos o dificultades para adquirir sensores, cables u otros componentes.</t>
   </si>
   <si>
     <t>Identificar componentes necesarios con anticipación y considerar alternativas compatibles</t>
   </si>
   <si>
-    <t>Sustituir temporalmente por un componente equivalente o ajustar las pruebas</t>
+    <t>Sustituir temporalmente por un componente equivalente o ajustar las pruebas.</t>
   </si>
   <si>
     <t>R-13</t>
@@ -310,142 +310,112 @@
     <t>R-16</t>
   </si>
   <si>
-    <t>Errores en la interfaz de usuario</t>
-  </si>
-  <si>
-    <t>Errores de diseño, navegación o validación de datos</t>
-  </si>
-  <si>
-    <t>Realizar pruebas de navegación, validación de campos y revisión de pantallas</t>
-  </si>
-  <si>
-    <t>Corregir la interfaz y repetir las pruebas afectadas</t>
+    <t>Dificultad para interpretar los estados de los espacios</t>
+  </si>
+  <si>
+    <t>Estados o indicadores visuales poco claros para el usuario.</t>
+  </si>
+  <si>
+    <t>Definir indicadores claros para disponible, ocupado, reservado y otros estados.</t>
+  </si>
+  <si>
+    <t>Ajustar colores, iconos, textos o distribución de la información.</t>
+  </si>
+  <si>
+    <t>Alberto / Santiago</t>
+  </si>
+  <si>
+    <t>R-17</t>
+  </si>
+  <si>
+    <t>Retraso en actividades del proyecto</t>
+  </si>
+  <si>
+    <t>Subestimación de tiempos, bloqueos técnicos o incumplimiento de tareas.</t>
+  </si>
+  <si>
+    <t>Dar seguimiento al cronograma, actualizar GitHub y reportar bloqueos oportunamente.</t>
+  </si>
+  <si>
+    <t>Reorganizar prioridades, reasignar tareas y actualizar el cronograma.</t>
+  </si>
+  <si>
+    <t>R-18</t>
+  </si>
+  <si>
+    <t>Errores en la configuración del entorno de desarrollo</t>
+  </si>
+  <si>
+    <t>Configuraciones diferentes entre equipos o dependencias incorrectas.</t>
+  </si>
+  <si>
+    <t>Documentar versiones, dependencias y configuración requerida.</t>
+  </si>
+  <si>
+    <t>Reinstalar/configurar el entorno siguiendo la documentación del proyecto.</t>
+  </si>
+  <si>
+    <t>R-19</t>
+  </si>
+  <si>
+    <t>Cambios en la interfaz durante el desarrollo</t>
+  </si>
+  <si>
+    <t>Ajustes derivados de pruebas, retroalimentación o mejoras de navegación.</t>
+  </si>
+  <si>
+    <t>Registrar los cambios y evaluar su impacto antes de implementarlos.</t>
+  </si>
+  <si>
+    <t>Reprogramar el cambio para una iteración posterior si afecta otras actividades.</t>
   </si>
   <si>
     <t>Alberto / Fernando</t>
   </si>
   <si>
-    <t>R-17</t>
-  </si>
-  <si>
-    <t>Consumo elevado de recursos en Raspberry Pi</t>
-  </si>
-  <si>
-    <t>Incremento de sensores, mensajes MQTT o procesos ejecutándose simultáneamente</t>
-  </si>
-  <si>
-    <t>Monitorear CPU, RAM y procesos durante las pruebas</t>
-  </si>
-  <si>
-    <t>Reducir frecuencia de actualización, optimizar procesos o reiniciar servicios</t>
-  </si>
-  <si>
-    <t>R-18</t>
-  </si>
-  <si>
-    <t>Dificultad para interpretar los estados de los espacios</t>
-  </si>
-  <si>
-    <t>Estados o indicadores visuales poco claros para el usuario</t>
-  </si>
-  <si>
-    <t>Definir indicadores claros para disponible, ocupado, reservado y otros estados</t>
-  </si>
-  <si>
-    <t>Ajustar colores, iconos, textos o distribución de la información</t>
-  </si>
-  <si>
-    <t>Alberto / Santiago</t>
-  </si>
-  <si>
-    <t>R-19</t>
-  </si>
-  <si>
-    <t>Retraso en actividades del proyecto</t>
-  </si>
-  <si>
-    <t>Subestimación de tiempos, bloqueos técnicos o incumplimiento de tareas.</t>
-  </si>
-  <si>
-    <t>Dar seguimiento al cronograma, actualizar GitHub Project y reportar bloqueos oportunamente.</t>
-  </si>
-  <si>
-    <t>Reorganizar prioridades, reasignar tareas y actualizar el cronograma.</t>
-  </si>
-  <si>
     <t>R-20</t>
   </si>
   <si>
-    <t>Errores en la configuración del entorno de desarrollo</t>
-  </si>
-  <si>
-    <t>Configuraciones diferentes entre equipos o dependencias incorrectas</t>
-  </si>
-  <si>
-    <t>Documentar versiones, dependencias y configuración requerida</t>
-  </si>
-  <si>
-    <t>Reinstalar/configurar el entorno siguiendo la documentación del proyecto</t>
+    <t>Incompatibilidad de la aplicación con algunos dispositivos</t>
+  </si>
+  <si>
+    <t>Diferencias de versiones, resolución o características del dispositivo.</t>
+  </si>
+  <si>
+    <t>Realizar pruebas en diferentes versiones y tamaños de pantalla.</t>
+  </si>
+  <si>
+    <t>Corregir problemas de compatibilidad y establecer versión mínima soportada.</t>
   </si>
   <si>
     <t>R-21</t>
   </si>
   <si>
-    <t>Cambios menores en la interfaz durante el desarrollo</t>
-  </si>
-  <si>
-    <t>Ajustes derivados de pruebas, retroalimentación o mejoras de navegación</t>
-  </si>
-  <si>
-    <t>Registrar los cambios y evaluar su impacto antes de implementarlos</t>
-  </si>
-  <si>
-    <t>Reprogramar el cambio para una iteración posterior si afecta otras actividades</t>
+    <t>Pérdida de información por falta de respaldos</t>
+  </si>
+  <si>
+    <t>Ausencia de copias de seguridad de la información almacenada.</t>
+  </si>
+  <si>
+    <t>Establecer respaldos periódicos de la base de datos y verificar su recuperación.</t>
+  </si>
+  <si>
+    <t>Restaurar la última copia disponible y recuperar los registros afectados.</t>
   </si>
   <si>
     <t>R-22</t>
   </si>
   <si>
-    <t>Incompatibilidad de la aplicación con algunos dispositivos</t>
-  </si>
-  <si>
-    <t>Diferencias de versiones, resolución o características del dispositivo</t>
-  </si>
-  <si>
-    <t>Realizar pruebas en diferentes versiones y tamaños de pantalla</t>
-  </si>
-  <si>
-    <t>Corregir problemas de compatibilidad y establecer versión mínima soportada</t>
-  </si>
-  <si>
-    <t>R-23</t>
-  </si>
-  <si>
-    <t>Pérdida de información por falta de respaldos</t>
-  </si>
-  <si>
-    <t>Ausencia de copias de seguridad de la información almacenada</t>
-  </si>
-  <si>
-    <t>Establecer respaldos periódicos de la base de datos y verificar su recuperación</t>
-  </si>
-  <si>
-    <t>Restaurar la última copia disponible y recuperar los registros afectados</t>
-  </si>
-  <si>
-    <t>R-24</t>
-  </si>
-  <si>
     <t>Pérdida o desorganización de evidencias y documentación</t>
   </si>
   <si>
-    <t>Archivos almacenados sin estructura o sin control de versiones</t>
-  </si>
-  <si>
-    <t>Mantener documentación y evidencias organizadas en el repositorio</t>
-  </si>
-  <si>
-    <t>Recuperar archivos desde GitHub, copias locales o registros disponibles y reorganizarlos</t>
+    <t>Archivos almacenados sin estructura o sin control de versiones.</t>
+  </si>
+  <si>
+    <t>Mantener documentación y evidencias organizadas en el repositorio.</t>
+  </si>
+  <si>
+    <t>Recuperar archivos desde GitHub, copias locales o registros disponibles y reorganizarlos.</t>
   </si>
 </sst>
 </file>
@@ -717,7 +687,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A4:M28" displayName="RiskTable" name="RiskTable" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A4:M26" displayName="RiskTable" name="RiskTable" id="1">
   <tableColumns count="13">
     <tableColumn name="ID" id="1"/>
     <tableColumn name="Riesgo / condición" id="2"/>
@@ -1021,11 +991,11 @@
         <v>5.0</v>
       </c>
       <c r="F5" s="7">
-        <f t="shared" ref="F5:F28" si="1">D5*E5</f>
+        <f t="shared" ref="F5:F26" si="1">D5*E5</f>
         <v>20</v>
       </c>
       <c r="G5" s="8" t="str">
-        <f t="shared" ref="G5:G28" si="2">IF(F5&gt;=15,"Alta",IF(F5&gt;=6,"Media","Baja"))</f>
+        <f t="shared" ref="G5:G26" si="2">IF(F5&gt;=15,"Alta",IF(F5&gt;=6,"Media","Baja"))</f>
         <v>Alta</v>
       </c>
       <c r="H5" s="9" t="s">
@@ -1660,14 +1630,14 @@
         <v>100</v>
       </c>
       <c r="D20" s="6">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="E20" s="6">
         <v>3.0</v>
       </c>
       <c r="F20" s="13">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G20" s="8" t="str">
         <f t="shared" si="2"/>
@@ -1696,25 +1666,25 @@
       <c r="A21" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="5" t="s">
         <v>106</v>
       </c>
       <c r="D21" s="6">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="E21" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="F21" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="F21" s="7">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G21" s="8" t="str">
         <f t="shared" si="2"/>
-        <v>Media</v>
+        <v>Alta</v>
       </c>
       <c r="H21" s="9" t="s">
         <v>107</v>
@@ -1723,7 +1693,7 @@
         <v>108</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="K21" s="8" t="s">
         <v>21</v>
@@ -1735,7 +1705,7 @@
         <v>46282.0</v>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22">
       <c r="A22" s="4" t="s">
         <v>109</v>
       </c>
@@ -1749,15 +1719,15 @@
         <v>2.0</v>
       </c>
       <c r="E22" s="6">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="F22" s="13">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G22" s="8" t="str">
         <f t="shared" si="2"/>
-        <v>Media</v>
+        <v>Baja</v>
       </c>
       <c r="H22" s="9" t="s">
         <v>112</v>
@@ -1766,7 +1736,7 @@
         <v>113</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>114</v>
+        <v>33</v>
       </c>
       <c r="K22" s="8" t="s">
         <v>21</v>
@@ -1778,38 +1748,38 @@
         <v>46282.0</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="C23" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>117</v>
-      </c>
       <c r="D23" s="6">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="E23" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="F23" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="F23" s="13">
         <f t="shared" si="1"/>
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G23" s="8" t="str">
         <f t="shared" si="2"/>
-        <v>Alta</v>
+        <v>Media</v>
       </c>
       <c r="H23" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="I23" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="I23" s="9" t="s">
+      <c r="J23" s="9" t="s">
         <v>119</v>
-      </c>
-      <c r="J23" s="9" t="s">
-        <v>77</v>
       </c>
       <c r="K23" s="8" t="s">
         <v>21</v>
@@ -1835,15 +1805,15 @@
         <v>2.0</v>
       </c>
       <c r="E24" s="6">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="F24" s="13">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G24" s="8" t="str">
         <f t="shared" si="2"/>
-        <v>Baja</v>
+        <v>Media</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>123</v>
@@ -1852,7 +1822,7 @@
         <v>124</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="K24" s="8" t="s">
         <v>21</v>
@@ -1878,15 +1848,15 @@
         <v>2.0</v>
       </c>
       <c r="E25" s="6">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="F25" s="13">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G25" s="8" t="str">
         <f t="shared" si="2"/>
-        <v>Baja</v>
+        <v>Media</v>
       </c>
       <c r="H25" s="9" t="s">
         <v>128</v>
@@ -1895,7 +1865,7 @@
         <v>129</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="K25" s="8" t="s">
         <v>21</v>
@@ -1938,7 +1908,7 @@
         <v>134</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="K26" s="8" t="s">
         <v>21</v>
@@ -1950,91 +1920,14 @@
         <v>46282.0</v>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="D27" s="6">
-        <v>2.0</v>
-      </c>
-      <c r="E27" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="F27" s="13">
-        <f t="shared" si="1"/>
-        <v>8</v>
-      </c>
-      <c r="G27" s="8" t="str">
-        <f t="shared" si="2"/>
-        <v>Media</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="I27" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="J27" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="K27" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="L27" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="M27" s="11">
-        <v>46282.0</v>
-      </c>
-    </row>
+    <row r="27" ht="15.75" customHeight="1"/>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="D28" s="6">
-        <v>2.0</v>
-      </c>
-      <c r="E28" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="F28" s="13">
-        <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="G28" s="8" t="str">
-        <f t="shared" si="2"/>
-        <v>Media</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="I28" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="J28" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="K28" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="L28" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="M28" s="11">
-        <v>46282.0</v>
-      </c>
+      <c r="C28" s="14"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="M28" s="16"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="C29" s="14"/>
@@ -2068,14 +1961,7 @@
       <c r="G32" s="15"/>
       <c r="M32" s="16"/>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="C33" s="14"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="15"/>
-      <c r="F33" s="15"/>
-      <c r="G33" s="15"/>
-      <c r="M33" s="16"/>
-    </row>
+    <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
     <row r="36" ht="15.75" customHeight="1"/>
@@ -2086,21 +1972,26 @@
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1"/>
-    <row r="44" ht="15.75" customHeight="1"/>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="B44" s="17"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="18"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="17"/>
+      <c r="I44" s="17"/>
+      <c r="J44" s="17"/>
+      <c r="K44" s="17"/>
+      <c r="L44" s="17"/>
+      <c r="M44" s="17"/>
+      <c r="N44" s="17"/>
+    </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="18"/>
-      <c r="F45" s="18"/>
-      <c r="G45" s="18"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="17"/>
+      <c r="E45" s="19"/>
+      <c r="F45" s="19"/>
+      <c r="G45" s="19"/>
+      <c r="N45" s="16"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="E46" s="19"/>
@@ -2150,12 +2041,7 @@
       <c r="G53" s="19"/>
       <c r="N53" s="16"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1">
-      <c r="E54" s="19"/>
-      <c r="F54" s="19"/>
-      <c r="G54" s="19"/>
-      <c r="N54" s="16"/>
-    </row>
+    <row r="54" ht="15.75" customHeight="1"/>
     <row r="55" ht="15.75" customHeight="1"/>
     <row r="56" ht="15.75" customHeight="1"/>
     <row r="57" ht="15.75" customHeight="1"/>
@@ -3092,29 +2978,28 @@
     <row r="988" ht="15.75" customHeight="1"/>
     <row r="989" ht="15.75" customHeight="1"/>
     <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:M2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G28">
+  <conditionalFormatting sqref="G5:G27">
     <cfRule type="expression" dxfId="5" priority="1">
       <formula>G5="Alta"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G5:G28">
+  <conditionalFormatting sqref="G5:G27">
     <cfRule type="expression" dxfId="6" priority="2">
       <formula>G5="Media"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G5:G28">
+  <conditionalFormatting sqref="G5:G27">
     <cfRule type="expression" dxfId="7" priority="3">
       <formula>G5="Baja"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="K5:K28">
+    <dataValidation type="list" allowBlank="1" sqref="K5:K26">
       <formula1>"Abierto,Mitigando,Materializado,Cerrado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>